<commit_message>
feat(auto): drop isolated single holes (P43/P47 now listed as pending survey), dedupe coincident holes, expose extrusion distance
</commit_message>
<xml_diff>
--- a/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008/3940平台 1008炮孔数据报告.xlsx
+++ b/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008/3940平台 1008炮孔数据报告.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -521,16 +521,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>1943.336</v>
+        <v>1595.433</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>5247.008</v>
+        <v>4307.67</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>1.204</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>63.192</v>
+        <v>51.879</v>
       </c>
     </row>
     <row r="4">
@@ -541,16 +541,16 @@
       </c>
       <c r="B4" s="6" t="n"/>
       <c r="C4" s="7" t="n">
-        <v>1943.336</v>
+        <v>1595.433</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>5247.008</v>
+        <v>4307.67</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>1.204</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>63.192</v>
+        <v>51.879</v>
       </c>
     </row>
     <row r="5">
@@ -563,16 +563,16 @@
         <v>2</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>1285.647</v>
+        <v>1108.44</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>3471.246</v>
+        <v>2992.788</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>0.729</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>25.31</v>
+        <v>21.821</v>
       </c>
     </row>
     <row r="6">
@@ -585,82 +585,72 @@
         <v>3</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>706.077</v>
+        <v>578.481</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>1906.408</v>
+        <v>1561.898</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>0.68</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>12.964</v>
+        <v>10.621</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>0.500-1.000</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>716.072</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>1933.394</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>0.6909999999999999</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>13.368</v>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>小计</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="7" t="n">
+        <v>1686.92</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>4554.685</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0.712</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>32.442</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>小计</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="7" t="n">
-        <v>2707.796</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>7311.048</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>0.706</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>51.642</v>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="9" t="n">
+        <v>3282.354</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>8862.355</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>0.951</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>84.322</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>合计</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="9" t="n">
-        <v>4651.132</v>
-      </c>
-      <c r="D9" s="9" t="n">
-        <v>12558.057</v>
-      </c>
-      <c r="E9" s="9" t="n">
-        <v>0.914</v>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>114.834</v>
-      </c>
+      <c r="A9" s="4" t="n"/>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n"/>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>炮孔品位统计（孔数）</t>
+        </is>
+      </c>
       <c r="B10" s="4" t="n"/>
       <c r="C10" s="5" t="n"/>
       <c r="D10" s="5" t="n"/>
@@ -668,66 +658,54 @@
       <c r="F10" s="5" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>炮孔品位统计（孔数）</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>≥3</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>1.5-3</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>1-1.5</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>≥3</t>
+          <t>0.5-1</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>1.5-3</t>
+          <t>&lt;0.5</t>
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>1-1.5</t>
+          <t>合计孔数</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>0.5-1</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>&lt;0.5</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>35</v>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>合计孔数</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n">
         <v>50</v>
       </c>
     </row>

</xml_diff>